<commit_message>
finished all technical debt for now. Commit before making pricing changes.
</commit_message>
<xml_diff>
--- a/KlimaChallenge_PM.xlsx
+++ b/KlimaChallenge_PM.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -796,7 +796,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Session 8 Complete  |  Date: 2026-03-15  |  Platform: React Native / Expo</t>
+          <t>Session 11 Complete  |  Date: 2026-03-16  |  Platform: React Native / Expo</t>
         </is>
       </c>
       <c r="B2" s="45" t="n"/>
@@ -807,6 +807,7 @@
       <c r="G2" s="45" t="n"/>
       <c r="H2" s="46" t="n"/>
     </row>
+    <row r="3"/>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -822,16 +823,22 @@
       <c r="H4" s="46" t="n"/>
     </row>
     <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="3" t="n">
-        <v>8</v>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Sessions Completed</t>
+        </is>
       </c>
       <c r="B5" s="46" t="n"/>
-      <c r="C5" s="4" t="n">
-        <v>43</v>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Features Shipped</t>
+        </is>
       </c>
       <c r="D5" s="46" t="n"/>
-      <c r="E5" s="5" t="n">
-        <v>11</v>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Backlog Items Left</t>
+        </is>
       </c>
       <c r="F5" s="46" t="n"/>
       <c r="G5" s="6" t="inlineStr">
@@ -848,37 +855,45 @@
       <c r="J5" s="46" t="n"/>
     </row>
     <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
+      <c r="A6" s="8" t="n">
+        <v>11</v>
       </c>
       <c r="B6" s="46" t="n"/>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
+      <c r="C6" s="8" t="n">
+        <v>33</v>
       </c>
       <c r="D6" s="46" t="n"/>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="F6" s="46" t="n"/>
+      <c r="G6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="46" t="n"/>
+      <c r="I6" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="J6" s="46" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="F6" s="46" t="n"/>
-      <c r="G6" s="8" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="H6" s="46" t="n"/>
-      <c r="I6" s="8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="J6" s="46" t="n"/>
-    </row>
+    </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
@@ -1178,6 +1193,70 @@
       <c r="F18" t="inlineStr">
         <is>
           <t>8 features; full gamification loop complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>S9</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Stats &amp; Insights screen (4 stat cards, KlimaTicket progress bar, WeeklyBarChart custom view, Transport Mix, Top Routes, CO2 long-press tooltip), FinancialOverview donut tappable -&gt; /stats, profile Stats &amp; Insights button -&gt; /stats</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>app/stats.tsx (new), components/ui/FinancialOverview.tsx, app/profile.tsx</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>3 features; no chart library (gifted-charts removed - Metro bundler bug); custom View-based bars</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Tech debt sprint: 9 items cleared. Memory files added to git repo.</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>constants/transport.ts (new), user.tsx, stats.tsx, TripRouteFields.tsx, QuickAddTripModal.tsx, user_styles.tsx, tripStorage.ts, .claude/memory/</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>All tech debt cleared. Transport colors centralised. useMemo, await fixes, dead code removed, light theme removed, debounce added.</t>
         </is>
       </c>
     </row>
@@ -1208,7 +1287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1240,7 +1319,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Priority-ordered remaining work  |  Updated 2026-03-15  |  Session 8 complete</t>
+          <t>Priority-ordered remaining work  |  Updated 2026-03-16  |  Session 11 complete</t>
         </is>
       </c>
       <c r="B2" s="45" t="n"/>
@@ -1465,7 +1544,7 @@
       </c>
       <c r="G7" s="16" t="inlineStr">
         <is>
-          <t>⬜ Todo</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="H7" s="16" t="inlineStr">
@@ -1475,7 +1554,7 @@
       </c>
       <c r="I7" s="16" t="inlineStr">
         <is>
-          <t>High visual impact for users</t>
+          <t>Completed S9 - app/stats.tsx; 4 stat cards; KlimaTicket progress bar; WeeklyBarChart (custom View, 8 ISO weeks); Transport Mix; Top Routes (top 5); CO2 factor 0.16 kg/km</t>
         </is>
       </c>
     </row>
@@ -1510,7 +1589,7 @@
       </c>
       <c r="G8" s="17" t="inlineStr">
         <is>
-          <t>⬜ Todo</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="H8" s="17" t="inlineStr">
@@ -1520,7 +1599,7 @@
       </c>
       <c r="I8" s="17" t="inlineStr">
         <is>
-          <t>Core value prop of app</t>
+          <t>Completed S9 - CO2 saved stat card (0.16 kg/km x distance); long-press tooltip with methodology</t>
         </is>
       </c>
     </row>
@@ -1555,7 +1634,7 @@
       </c>
       <c r="G9" s="17" t="inlineStr">
         <is>
-          <t>⬜ Todo</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="H9" s="17" t="inlineStr">
@@ -1565,7 +1644,7 @@
       </c>
       <c r="I9" s="17" t="inlineStr">
         <is>
-          <t>Pairs with Stats screen</t>
+          <t>Completed S9 - Transport Mix (horizontal bars, %) + Top Routes (ranked top 5) + avg cost/trip + total distance</t>
         </is>
       </c>
     </row>
@@ -1690,7 +1769,7 @@
       </c>
       <c r="G12" s="12" t="inlineStr">
         <is>
-          <t>⬜ Todo</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="H12" s="12" t="inlineStr">
@@ -1700,7 +1779,7 @@
       </c>
       <c r="I12" s="12" t="inlineStr">
         <is>
-          <t>Easy perf win</t>
+          <t>useMemo([trips]) in user.tsx</t>
         </is>
       </c>
     </row>
@@ -1735,7 +1814,7 @@
       </c>
       <c r="G13" s="12" t="inlineStr">
         <is>
-          <t>⬜ Todo</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="H13" s="12" t="inlineStr">
@@ -1745,7 +1824,7 @@
       </c>
       <c r="I13" s="12" t="inlineStr">
         <is>
-          <t>DRY principle</t>
+          <t>constants/transport.ts — TRANSPORT_COLOR + transportIcon()</t>
         </is>
       </c>
     </row>
@@ -1780,7 +1859,7 @@
       </c>
       <c r="G14" s="17" t="inlineStr">
         <is>
-          <t>⬜ Todo</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="H14" s="17" t="inlineStr">
@@ -1790,7 +1869,7 @@
       </c>
       <c r="I14" s="17" t="inlineStr">
         <is>
-          <t>Prevents potential date-related runtime errors</t>
+          <t>Already resolved - loadTrips() does date: new Date(trip.date) on parse. Closed S9 audit.</t>
         </is>
       </c>
     </row>
@@ -1825,7 +1904,7 @@
       </c>
       <c r="G15" s="12" t="inlineStr">
         <is>
-          <t>⬜ Todo</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="H15" s="12" t="inlineStr">
@@ -1833,7 +1912,11 @@
           <t>Any</t>
         </is>
       </c>
-      <c r="I15" s="12" t="inlineStr"/>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>400ms debounce via searchDebounceRef in QuickAddTripModal</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="45" customHeight="1">
       <c r="A16" s="15" t="n">
@@ -2368,6 +2451,366 @@
       <c r="I27" t="inlineStr">
         <is>
           <t>Completed S8 - MainQuestFeaturedCard component in quests.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>25</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Tech Debt</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Memoize recentPlaces</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>recentPlaces IIFE computed inline on every render in user.tsx (same pattern as computeFavorites). Wrap in useMemo([trips]).</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>🔵 Low</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>XS (30m)</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>S10</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>useMemo([trips]) in user.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>26</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Tech Debt</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Fix Floating checkMainQuest Promise</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>checkMainQuest() called without await in handleFavoritePress and handleQuickAddSubmit. Errors silently swallowed.</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>🟡 Medium</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>XS (15m)</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>S10</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>await added in handleFavoritePress + handleQuickAddSubmit</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>27</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Tech Debt</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Remove getTripById Dead Code</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>getTripById() in tripStorage.ts is never called anywhere in the codebase. Dead code from old trip detail screen.</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>🔵 Low</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>XS (5m)</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>S10</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>getTripById removed from tripStorage.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>28</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Tech Debt</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Verify / Remove Light Theme in TripRouteFields</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>TripRouteFields has full light-theme StyleSheet. QuickAdd was converted to dark (S7) — verify theme=light is unused; remove dead styles.</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>🔵 Low</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>XS (30m)</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>S10</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>theme prop + light styles removed from TripRouteFields</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>29</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Tech Debt</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Merge screenStyles into user_styles.tsx</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>user.tsx has a separate screenStyles StyleSheet with a single entry (root: flex 1). Should live in user_styles.tsx.</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>🔵 Low</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>XS (5m)</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>S10</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>root style moved to user_styles.tsx; screenStyles removed</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>30</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Tech Debt</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Hoist typeIcon() in stats.tsx</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>typeIcon() helper defined after the component that uses it in stats.tsx. Hoist above StatsScreen.</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>🔵 Low</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>XS (5m)</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>S10</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>typeIcon() moved to constants/transport.ts as transportIcon()</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>31</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Tech Debt</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Add eslint-disable to TripRouteFields useEffect</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>useEffect intentionally omits cost/onCostChange from deps (mount guard pattern). Add eslint-disable-next-line comment to document intent.</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>🔵 Low</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>XS (5m)</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>S10</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>eslint-disable comment added above useEffect mount guard</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>32</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>PM Updater Script</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Persistent Python helper (pm_updater.py) with PMUpdater class to update KlimaChallenge_PM.xlsx. Replaces one-off scripts written each session. Methods: add_session_row, mark_backlog_done, add_backlog_item, add_feature, update_milestone, add_velocity_row, update_sprint_plan, add_arch_session.</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>🔵 Low</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>S (1-2h)</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>S10</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Completed S10 - PMUpdater class with 14 methods; dynamic row-finding; idempotent (skip if already exists); __main__ template for Claude to fill each session.</t>
         </is>
       </c>
     </row>
@@ -2386,7 +2829,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2668,22 +3111,22 @@
       </c>
       <c r="B11" s="21" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="C11" s="21" t="inlineStr">
         <is>
-          <t>⬜ Planned</t>
+          <t>✅ Complete</t>
         </is>
       </c>
       <c r="D11" s="22" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="E11" s="21" t="inlineStr">
         <is>
-          <t>Stats screen with charts, CO2 display, trip statistics summary, pricing API research</t>
+          <t>Stats screen with charts, CO2 display, trip statistics, transport mix, top routes</t>
         </is>
       </c>
       <c r="F11" s="21" t="inlineStr">
@@ -2693,7 +3136,7 @@
       </c>
       <c r="G11" s="21" t="inlineStr">
         <is>
-          <t>Sessions 8-9</t>
+          <t>Sessions 8-9; complete end of S9</t>
         </is>
       </c>
     </row>
@@ -2734,6 +3177,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="8" customHeight="1"/>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
@@ -2988,7 +3432,32 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="8" customHeight="1"/>
+    <row r="25" ht="8" customHeight="1">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>S9</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Mar 16</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>3</v>
+      </c>
+      <c r="D25" t="n">
+        <v>46</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Stats &amp; Insights</t>
+        </is>
+      </c>
+    </row>
     <row r="26"/>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
@@ -3137,17 +3606,17 @@
       </c>
       <c r="E31" s="11" t="inlineStr">
         <is>
-          <t>Heavy</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F31" s="11" t="inlineStr">
         <is>
-          <t>🟡 Medium</t>
+          <t>🟢 Low</t>
         </is>
       </c>
       <c r="G31" s="11" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Completed - 3 features; gifted-charts removed (Metro bug); custom View-based bars</t>
         </is>
       </c>
     </row>
@@ -3164,12 +3633,12 @@
       </c>
       <c r="C32" s="19" t="inlineStr">
         <is>
-          <t>Pricing &amp; Polish</t>
+          <t>Tech Debt + Optimization</t>
         </is>
       </c>
       <c r="D32" s="19" t="inlineStr">
         <is>
-          <t>Pricing API research, more route prices, debounce, memoize, transport constants</t>
+          <t>useMemo (computeFavorites + recentPlaces), centralise+fix transport constants, fix floating promise, remove dead code, debounce OBB, more route prices</t>
         </is>
       </c>
       <c r="E32" s="19" t="inlineStr">
@@ -3211,7 +3680,7 @@
       </c>
       <c r="E33" s="25" t="inlineStr">
         <is>
-          <t>Light-Medium</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F33" s="25" t="inlineStr">
@@ -3221,7 +3690,7 @@
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -3259,6 +3728,32 @@
       <c r="G34" s="19" t="inlineStr">
         <is>
           <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Mar 16</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" t="n">
+        <v>33</v>
+      </c>
+      <c r="E35" t="n">
+        <v>9</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Tech Debt</t>
         </is>
       </c>
     </row>
@@ -3280,7 +3775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3716,7 +4211,7 @@
       </c>
       <c r="B17" s="27" t="inlineStr">
         <is>
-          <t>(planned)</t>
+          <t>Custom View-based bars (no library)</t>
         </is>
       </c>
       <c r="C17" s="27" t="inlineStr">
@@ -3726,17 +4221,17 @@
       </c>
       <c r="D17" s="27" t="inlineStr">
         <is>
-          <t>Stats screen visualisations</t>
+          <t>Stats screen weekly bar chart, transport mix bars, progress bars</t>
         </is>
       </c>
       <c r="E17" s="27" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>app/stats.tsx</t>
         </is>
       </c>
       <c r="F17" s="27" t="inlineStr">
         <is>
-          <t>Candidate: react-native-gifted-charts or Victory Native</t>
+          <t>react-native-gifted-charts tried S9 and removed (Metro bundler resolution bug); custom Views sufficient</t>
         </is>
       </c>
     </row>
@@ -3882,7 +4377,7 @@
       </c>
       <c r="D26" s="21" t="inlineStr">
         <is>
-          <t>⚠️ Normalise date to Date object in loadTrips() — tech debt</t>
+          <t>RESOLVED S9 — loadTrips() does date: new Date(trip.date) on parse. Tech debt closed.</t>
         </is>
       </c>
     </row>
@@ -4031,6 +4526,70 @@
       <c r="F33" t="inlineStr">
         <is>
           <t>8 features; full gamification loop</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>S9</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>app/stats.tsx (new)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>No chart library — custom View WeeklyBarChart to avoid Metro bundler issues; CO2 factor 0.16 kg/km (car 0.21 - PT 0.05); ISO week helper for 8-week window; TRANSPORT_COLOR map added in stats.tsx (inconsistency vs user.tsx TRANSPORT_ACCENT — tech debt #10)</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>None added</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>3 features; stats screen complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>constants/transport.ts, .claude/memory/ (project memory in git)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Canonical transport colors: Bus=blue.mid, Train=green.mid, Tram=red.light, Subway=green.dark. Memory files now version-controlled in .claude/memory/.</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>None added</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Pure tech debt session. All 9 remaining debt items resolved.</t>
         </is>
       </c>
     </row>
@@ -4053,7 +4612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -5856,6 +6415,166 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>44</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Stats &amp; Insights Screen</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>S9</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>app/stats.tsx (new)</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>4 stat cards (trips, distance, CO2 saved, avg cost/trip); KlimaTicket progress bar (% + remaining); WeeklyBarChart (custom View, 8 ISO weeks, no library); Transport Mix (horizontal bars, %, color-coded); Top Routes (ranked list top 5); CO2 long-press tooltip; empty state; back button</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>45</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Stats Entry — FinancialOverview Donut</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>S9</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>components/ui/FinancialOverview.tsx</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Added onStatsPress prop; SVG donut circle wrapped in TouchableOpacity; tapping navigates to /stats from main screen</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>46</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Stats Entry — Profile Button</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>UX</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>S9</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>app/profile.tsx</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Stats &amp; Insights button in profile screen; navigates to /stats</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>47</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>PM Updater Script</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>S10</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>pm_updater.py (new)</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>PMUpdater class with 14 methods covering all 5 Excel sheets. Dynamic row-finding (no hardcoded positions). Idempotent operations (skip if already exists). __main__ template block for Claude to fill at session end. Reduces per-session Excel update time from ~15min to ~2min.</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:H2"/>

</xml_diff>

<commit_message>
Added new items to backlog.
</commit_message>
<xml_diff>
--- a/KlimaChallenge_PM.xlsx
+++ b/KlimaChallenge_PM.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -864,7 +864,7 @@
       </c>
       <c r="D6" s="46" t="n"/>
       <c r="E6" s="8" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F6" s="46" t="n"/>
       <c r="G6" s="8" t="n">
@@ -872,19 +872,19 @@
       </c>
       <c r="H6" s="46" t="n"/>
       <c r="I6" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J6" s="46" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>35</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1287,6 +1287,38 @@
         </is>
       </c>
       <c r="F21" t="inlineStr">
+        <is>
+          <t>3 compounding bugs in Delete All Trips: RNGH gestures dead in RN Modal (fixed with absolute overlay), runOnJS broken on web (fixed with .runOnJS(true)+setTimeout), wrong storage key @trips vs @travelapp_trips + initialTrips fallback (fixed with saveTrips([])).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>KlimaTicket presets overhaul (6 nationwide + 20 regional, real 2026 prices). Delete All Trips with slide-to-confirm. Bug fixes: typeIcon crash, Expo Router route warning, RNGH-in-Modal, wrong AsyncStorage key.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>profile.tsx, stats.tsx, app/(tabs)/user.tsx, app/(tabs)/_user_styles.tsx (renamed)</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
         <is>
           <t>3 compounding bugs in Delete All Trips: RNGH gestures dead in RN Modal (fixed with absolute overlay), runOnJS broken on web (fixed with .runOnJS(true)+setTimeout), wrong storage key @trips vs @travelapp_trips + initialTrips fallback (fixed with saveTrips([])).</t>
         </is>
@@ -1319,7 +1351,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2981,6 +3013,231 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>36</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Delete All Trips — reset quests/achievements too</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>handleDeleteAllTrips clears trips+XP+mainQuestCelebrated but not @claimedQuests, @claimedAchievements, @dailyQuestSelection, @weeklyQuestSelection. User who resets sees stale claimed state.</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>🔴 Critical</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>XS (30m)</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>⬜ Todo</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>S13</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Add removeItem calls for all 4 keys in handleDeleteAllTrips in profile.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>37</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Remove initialTrips demo data fallback</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>loadTrips() in tripStorage.ts returns 10 hardcoded dummy trips when key missing. New users see fake data. Pre-prod blocker.</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>🔴 Critical</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>XS (15m)</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>⬜ Todo</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>S13</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Change fallback from `return initialTrips` to `return []` in tripStorage.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>38</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>UX</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Profile dropdown — close on outside tap</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>KlimaTicket dropdown in profile stays open when user taps outside. Should dismiss.</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>🟡 Medium</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>XS (30m)</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>⬜ Todo</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Wrap screen in TouchableWithoutFeedback or use onStartShouldSetResponder pattern</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>39</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Cloud sync for trips (Supabase)</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Trips stored in AsyncStorage only — new device login starts from scratch. Sync to Supabase trips table.</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>🟠 High</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>L (1-2d)</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>⬜ Todo</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Requires Supabase trips table schema, upsert on save, fetch on login</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>40</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Trip export / CSV download</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Allow users to export all trips as CSV for tax/Jobticket purposes.</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>🔵 Low</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>S (2-4h)</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>⬜ Todo</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Use expo-sharing + expo-file-system to write and share CSV</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
@@ -2996,7 +3253,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3945,6 +4202,32 @@
         <v>0</v>
       </c>
       <c r="F36" t="inlineStr">
+        <is>
+          <t>Feature + Bug Fix</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Mar 16</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>2</v>
+      </c>
+      <c r="D37" t="n">
+        <v>35</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="inlineStr">
         <is>
           <t>Feature + Bug Fix</t>
         </is>
@@ -3968,7 +4251,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4813,6 +5096,38 @@
         </is>
       </c>
       <c r="F36" t="inlineStr">
+        <is>
+          <t>3 compounding bugs resolved in Delete All Trips feature. STORAGE_KEY=@travelapp_trips (not @trips). loadTrips() returns initialTrips when key missing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>None (profile.tsx, user.tsx, stats.tsx modified)</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>RNGH gestures do NOT work inside RN Modal on mobile — use absolute-positioned View overlay instead. saveTrips([]) to clear trips (removeItem would trigger initialTrips fallback). useFocusEffect reloads trips+XP on every screen focus.</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>None added</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
         <is>
           <t>3 compounding bugs resolved in Delete All Trips feature. STORAGE_KEY=@travelapp_trips (not @trips). loadTrips() returns initialTrips when key missing.</t>
         </is>

</xml_diff>